<commit_message>
Deployed 91e13e6b with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/en/Manual/source/tab/parameters.xlsx
+++ b/en/Manual/source/tab/parameters.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="21"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="35"/>
   </bookViews>
   <sheets>
     <sheet name="TGZ-D-48-13_26" sheetId="1" state="visible" r:id="rId3"/>
@@ -43,15 +43,16 @@
     <sheet name="TGZ-D-560-30_50" sheetId="33" state="visible" r:id="rId35"/>
     <sheet name="TGS-320-10_15" sheetId="34" state="visible" r:id="rId36"/>
     <sheet name="TGS-560-25_50" sheetId="35" state="visible" r:id="rId37"/>
-    <sheet name="TGS-560-50_100" sheetId="36" state="visible" r:id="rId38"/>
-    <sheet name="TGMmini" sheetId="37" state="visible" r:id="rId39"/>
-    <sheet name="TGMcontroller" sheetId="38" state="visible" r:id="rId40"/>
-    <sheet name="TGZpMotion" sheetId="39" state="visible" r:id="rId41"/>
-    <sheet name="X8_commonHW_DI_tab" sheetId="40" state="visible" r:id="rId42"/>
-    <sheet name="X8_commonHW_DI_RI_tab" sheetId="41" state="visible" r:id="rId43"/>
-    <sheet name="X8_commonHW_DO_tab" sheetId="42" state="visible" r:id="rId44"/>
-    <sheet name="X8_commonHW_AI_tab" sheetId="43" state="visible" r:id="rId45"/>
-    <sheet name="TGmonitor7" sheetId="44" state="visible" r:id="rId46"/>
+    <sheet name="TGZ-D-48-50_100-UNIR-RI" sheetId="36" state="visible" r:id="rId38"/>
+    <sheet name="TGS-560-50_100" sheetId="37" state="visible" r:id="rId39"/>
+    <sheet name="TGMmini" sheetId="38" state="visible" r:id="rId40"/>
+    <sheet name="TGMcontroller" sheetId="39" state="visible" r:id="rId41"/>
+    <sheet name="TGZpMotion" sheetId="40" state="visible" r:id="rId42"/>
+    <sheet name="X8_commonHW_DI_tab" sheetId="41" state="visible" r:id="rId43"/>
+    <sheet name="X8_commonHW_DI_RI_tab" sheetId="42" state="visible" r:id="rId44"/>
+    <sheet name="X8_commonHW_DO_tab" sheetId="43" state="visible" r:id="rId45"/>
+    <sheet name="X8_commonHW_AI_tab" sheetId="44" state="visible" r:id="rId46"/>
+    <sheet name="TGmonitor7" sheetId="45" state="visible" r:id="rId47"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -63,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2191" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2251" uniqueCount="346">
   <si>
     <t xml:space="preserve">POWER SUPPLY</t>
   </si>
@@ -774,6 +775,9 @@
   </si>
   <si>
     <t xml:space="preserve">1 x 3pin WEIDMÜLLER BLZ 7.62HP/03/180F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 x 5pin WEIDMÜLLER  BCZ 3.81/05/180F</t>
   </si>
   <si>
     <t xml:space="preserve">3 x 400 VAC/50Hz 63A</t>
@@ -1258,37 +1262,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -4677,7 +4681,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="42.85"/>
@@ -4845,74 +4849,82 @@
         <v>77</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>32</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B28" s="2" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>140</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B33" s="2" t="s">
         <v>141</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="2" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="B35" s="4" t="s">
+      <c r="B36" s="4" t="s">
         <v>147</v>
       </c>
     </row>
@@ -8196,12 +8208,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="42.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="45.61"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="2" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="52.92"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8217,212 +8228,244 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>168</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>192</v>
+        <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="C3" s="2"/>
+        <v>5</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>194</v>
+        <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C4" s="2"/>
+        <v>48</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>195</v>
+        <v>8</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="C5" s="2"/>
+        <v>49</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>197</v>
+        <v>10</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C6" s="2"/>
+        <v>50</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>199</v>
+        <v>12</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C7" s="2"/>
+        <v>51</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="C8" s="2"/>
+        <v>52</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>201</v>
+        <v>16</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="C9" s="2"/>
+        <v>17</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C10" s="2"/>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="C11" s="2"/>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>18</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>239</v>
+        <v>20</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="C12" s="2"/>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" s="2"/>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>21</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C14" s="2"/>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>23</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>210</v>
+        <v>68</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>211</v>
+        <v>69</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="B20" s="4"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>214</v>
+        <v>76</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>231</v>
+        <v>100</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>241</v>
-      </c>
-    </row>
+        <v>85</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>216</v>
+        <v>30</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>218</v>
+        <v>31</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>219</v>
+        <v>32</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>242</v>
+        <v>61</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>219</v>
+        <v>34</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>244</v>
-      </c>
+      <c r="A29" s="2"/>
+      <c r="B29" s="2"/>
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="2"/>
+      <c r="B35" s="2"/>
+    </row>
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="2"/>
+      <c r="B36" s="2"/>
+    </row>
+    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="2"/>
+      <c r="B37" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -8440,7 +8483,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="42.22"/>
@@ -8458,73 +8501,78 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>245</v>
+        <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="C2" s="2"/>
+        <v>168</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>247</v>
+        <v>192</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="C3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>249</v>
+        <v>194</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>246</v>
+        <v>49</v>
       </c>
       <c r="C4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>19</v>
+        <v>195</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>222</v>
       </c>
       <c r="C5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="C6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>20</v>
+        <v>199</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="C7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>250</v>
+        <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>251</v>
+        <v>239</v>
       </c>
       <c r="C8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>252</v>
+        <v>201</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>253</v>
+        <v>226</v>
       </c>
       <c r="C9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>21</v>
+        <v>203</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>1</v>
@@ -8533,82 +8581,134 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>254</v>
+        <v>205</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>255</v>
+        <v>184</v>
       </c>
       <c r="C11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>256</v>
+        <v>240</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>257</v>
+        <v>241</v>
       </c>
       <c r="C12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>258</v>
+        <v>16</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>259</v>
+        <v>17</v>
       </c>
       <c r="C13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="C14" s="2"/>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C15" s="2"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>260</v>
+        <v>209</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="C16" s="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>211</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>263</v>
+        <v>211</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>264</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>265</v>
+        <v>61</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>266</v>
+        <v>213</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>245</v>
       </c>
     </row>
   </sheetData>
@@ -8645,28 +8745,28 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C4" s="2"/>
     </row>
@@ -8693,19 +8793,19 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>23</v>
+        <v>251</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>24</v>
+        <v>252</v>
       </c>
       <c r="C8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>25</v>
+        <v>253</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>26</v>
+        <v>254</v>
       </c>
       <c r="C9" s="2"/>
     </row>
@@ -8720,84 +8820,82 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="C11" s="2"/>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="C11" s="2"/>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="2" t="s">
+        <v>258</v>
+      </c>
       <c r="C12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="C13" s="2"/>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C14" s="2"/>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C13" s="2"/>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="C14" s="2"/>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="2" t="s">
+        <v>1</v>
+      </c>
       <c r="C15" s="2"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>214</v>
+        <v>261</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>1</v>
+        <v>262</v>
       </c>
       <c r="C16" s="2"/>
-    </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>39</v>
-      </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>21</v>
+        <v>214</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>264</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>28</v>
+        <v>263</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>104</v>
+        <v>264</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>110</v>
+        <v>265</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>44</v>
+        <v>266</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>111</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -8816,7 +8914,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="42.22"/>
@@ -8834,28 +8932,28 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C4" s="2"/>
     </row>
@@ -8909,10 +9007,10 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C11" s="2"/>
     </row>
@@ -8930,10 +9028,10 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C14" s="2"/>
     </row>
@@ -8951,18 +9049,42 @@
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>21</v>
+        <v>263</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>264</v>
+        <v>39</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B19" s="2" t="s">
         <v>104</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -9215,6 +9337,171 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="42.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="45.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="2" width="11.53"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="2"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="2"/>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" s="2"/>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="C11" s="2"/>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C12" s="2"/>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13" s="2"/>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="C14" s="2"/>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C15" s="2"/>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C16" s="2"/>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:K11"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -9231,107 +9518,107 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9339,16 +9626,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>24</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>2.05</v>
@@ -9374,16 +9661,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>24</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>2.05</v>
@@ -9409,16 +9696,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>24</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>2.05</v>
@@ -9444,16 +9731,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>24</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F7" s="2" t="n">
         <v>2.05</v>
@@ -9479,16 +9766,16 @@
         <v>5</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>24</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F8" s="2" t="n">
         <v>2.05</v>
@@ -9514,16 +9801,16 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>24</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>2.05</v>
@@ -9549,16 +9836,16 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>24</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>1.25</v>
@@ -9584,16 +9871,16 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>24</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F11" s="2" t="n">
         <v>1.25</v>
@@ -9625,7 +9912,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -9645,98 +9932,98 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9744,10 +10031,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>24</v>
@@ -9776,10 +10063,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>24</v>
@@ -9808,10 +10095,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>24</v>
@@ -9840,10 +10127,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>24</v>
@@ -9872,10 +10159,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>24</v>
@@ -9904,10 +10191,10 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>24</v>
@@ -9936,10 +10223,10 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>24</v>
@@ -9968,10 +10255,10 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>24</v>
@@ -10006,7 +10293,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -10026,89 +10313,89 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10128,7 +10415,7 @@
         <v>0.5</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>300</v>
@@ -10157,7 +10444,7 @@
         <v>0.5</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>300</v>
@@ -10186,7 +10473,7 @@
         <v>0.5</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>300</v>
@@ -10215,7 +10502,7 @@
         <v>0.5</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>300</v>
@@ -10244,7 +10531,7 @@
         <v>0.5</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>300</v>
@@ -10273,7 +10560,7 @@
         <v>0.5</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>300</v>
@@ -10283,101 +10570,6 @@
       </c>
       <c r="I9" s="2" t="n">
         <v>10</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="10.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="20.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="27.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="30.24"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>318</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>279</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>320</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>321</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
-        <v>290</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>291</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -10396,6 +10588,101 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="10.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="20.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="27.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="30.24"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:B18"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -10414,18 +10701,18 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -10439,32 +10726,32 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>1</v>
@@ -10472,66 +10759,66 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
   </sheetData>

</xml_diff>